<commit_message>
Numerología v0.1: hoja opcional con el nombre completo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/referencias/numerologia/Numerologia-Destiny-propuesta-v0.xlsx
+++ b/docs/referencias/numerologia/Numerologia-Destiny-propuesta-v0.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Matriz" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Parámetros" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Calculadora" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Con nombre" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -608,7 +609,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>• Si preferís otro método (otros números, nombre completo, otra forma de comparar), contame y lo armo.</t>
+          <t>• Si preferís otro método (otros números, otra forma de comparar), contame y lo armo.</t>
         </is>
       </c>
     </row>
@@ -616,14 +617,52 @@
       <c r="A23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Los valores de este borrador salen de las reglas clásicas de la numerología (grupos 1-5-7, 3-6-9, 2-4-8 y</t>
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>Opcional, con el nombre completo de nacimiento (hoja Con nombre):</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
+        <is>
+          <t>• Expresión (todas las letras), Alma (vocales) y Personalidad (consonantes), con la tabla pitagórica (A=1 … I=9, J=1 …).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>• Alma → Afecto, Personalidad → Química, Expresión → Comunicación y Compromiso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>• Se mezcla con lo de la fecha según el Peso del nombre (hoja Parámetros, 50 % de arranque).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>• Sería opcional en la app: el nombre que guardamos hoy es el apodo del perfil, que no sirve para esto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Los valores de este borrador salen de las reglas clásicas de la numerología (grupos 1-5-7, 3-6-9, 2-4-8 y</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>combinaciones en tensión como 4-5 y 1-8). Son un punto de partida: el modelo final lo definís vos.</t>
         </is>
@@ -1318,6 +1357,16 @@
       </c>
       <c r="B3" s="3" t="n">
         <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Peso del nombre, si se carga (hoja Con nombre)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="5">
@@ -1945,4 +1994,478 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col hidden="1" width="13" customWidth="1" min="10" max="10"/>
+    <col hidden="1" width="13" customWidth="1" min="11" max="11"/>
+    <col hidden="1" width="13" customWidth="1" min="12" max="12"/>
+    <col hidden="1" width="13" customWidth="1" min="13" max="13"/>
+    <col hidden="1" width="13" customWidth="1" min="14" max="14"/>
+    <col hidden="1" width="13" customWidth="1" min="15" max="15"/>
+    <col hidden="1" width="13" customWidth="1" min="16" max="16"/>
+    <col hidden="1" width="13" customWidth="1" min="17" max="17"/>
+    <col hidden="1" width="13" customWidth="1" min="18" max="18"/>
+    <col hidden="1" width="13" customWidth="1" min="19" max="19"/>
+    <col hidden="1" width="13" customWidth="1" min="20" max="20"/>
+    <col hidden="1" width="13" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Opcional: con el nombre completo de nacimiento (el del acta). Poné los nombres en las celdas amarillas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Las fechas son las de la hoja Calculadora. Tildes y ñ se leen como la letra sin tilde y N; la Y cuenta como consonante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Persona A</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Persona B</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Nombre completo de nacimiento</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>María Laura Gómez</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Juan Pablo Ruiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Expresión</t>
+        </is>
+      </c>
+      <c r="B5" s="1">
+        <f>L35</f>
+        <v/>
+      </c>
+      <c r="C5" s="1">
+        <f>R35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="B6" s="1">
+        <f>L36</f>
+        <v/>
+      </c>
+      <c r="C6" s="1">
+        <f>R36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Personalidad</t>
+        </is>
+      </c>
+      <c r="B7" s="1">
+        <f>L37</f>
+        <v/>
+      </c>
+      <c r="C7" s="1">
+        <f>R37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Expresión (base)</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>IF(B5=11,2,IF(B5=22,4,IF(B5=33,6,B5)))</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>IF(C5=11,2,IF(C5=22,4,IF(C5=33,6,C5)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Alma (base)</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>IF(B6=11,2,IF(B6=22,4,IF(B6=33,6,B6)))</f>
+        <v/>
+      </c>
+      <c r="C9">
+        <f>IF(C6=11,2,IF(C6=22,4,IF(C6=33,6,C6)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Personalidad (base)</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>IF(B7=11,2,IF(B7=22,4,IF(B7=33,6,B7)))</f>
+        <v/>
+      </c>
+      <c r="C10">
+        <f>IF(C7=11,2,IF(C7=22,4,IF(C7=33,6,C7)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Eje</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Con la fecha</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Con el nombre</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Combinado</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>Química (Personalidad)</t>
+        </is>
+      </c>
+      <c r="B13" s="7">
+        <f>Calculadora!D17</f>
+        <v/>
+      </c>
+      <c r="C13" s="7">
+        <f>MAX(0,MIN(100,INDEX(Matriz!$B$3:$J$11,$B$10,$C$10)+Parámetros!$B$3*((INDEX(Números!$C$2:$C$10,$B$10)+INDEX(Números!$C$2:$C$10,$C$10))/2-50)/50))</f>
+        <v/>
+      </c>
+      <c r="D13" s="8">
+        <f>(1-Parámetros!$B$4)*B13+Parámetros!$B$4*C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Afecto (Alma)</t>
+        </is>
+      </c>
+      <c r="B14" s="7">
+        <f>Calculadora!D18</f>
+        <v/>
+      </c>
+      <c r="C14" s="7">
+        <f>MAX(0,MIN(100,INDEX(Matriz!$B$3:$J$11,$B$9,$C$9)+Parámetros!$B$3*((INDEX(Números!$D$2:$D$10,$B$9)+INDEX(Números!$D$2:$D$10,$C$9))/2-50)/50))</f>
+        <v/>
+      </c>
+      <c r="D14" s="8">
+        <f>(1-Parámetros!$B$4)*B14+Parámetros!$B$4*C14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>Comunicación (Expresión)</t>
+        </is>
+      </c>
+      <c r="B15" s="7">
+        <f>Calculadora!D19</f>
+        <v/>
+      </c>
+      <c r="C15" s="7">
+        <f>MAX(0,MIN(100,INDEX(Matriz!$B$3:$J$11,$B$8,$C$8)+Parámetros!$B$3*((INDEX(Números!$E$2:$E$10,$B$8)+INDEX(Números!$E$2:$E$10,$C$8))/2-50)/50))</f>
+        <v/>
+      </c>
+      <c r="D15" s="8">
+        <f>(1-Parámetros!$B$4)*B15+Parámetros!$B$4*C15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>Compromiso (Expresión)</t>
+        </is>
+      </c>
+      <c r="B16" s="7">
+        <f>Calculadora!D20</f>
+        <v/>
+      </c>
+      <c r="C16" s="7">
+        <f>MAX(0,MIN(100,INDEX(Matriz!$B$3:$J$11,$B$8,$C$8)+Parámetros!$B$3*((INDEX(Números!$F$2:$F$10,$B$8)+INDEX(Números!$F$2:$F$10,$C$8))/2-50)/50))</f>
+        <v/>
+      </c>
+      <c r="D16" s="8">
+        <f>(1-Parámetros!$B$4)*B16+Parámetros!$B$4*C16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Vínculo</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Solo fecha</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Con nombre</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>Pareja</t>
+        </is>
+      </c>
+      <c r="B19" s="7">
+        <f>Calculadora!B24</f>
+        <v/>
+      </c>
+      <c r="C19" s="8">
+        <f>D13*Parámetros!B6+D14*Parámetros!C6+D15*Parámetros!D6+D16*Parámetros!E6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>Amistad</t>
+        </is>
+      </c>
+      <c r="B20" s="7">
+        <f>Calculadora!B25</f>
+        <v/>
+      </c>
+      <c r="C20" s="8">
+        <f>D13*Parámetros!B7+D14*Parámetros!C7+D15*Parámetros!D7+D16*Parámetros!E7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>Trabajo</t>
+        </is>
+      </c>
+      <c r="B21" s="7">
+        <f>Calculadora!B26</f>
+        <v/>
+      </c>
+      <c r="C21" s="8">
+        <f>D13*Parámetros!B8+D14*Parámetros!C8+D15*Parámetros!D8+D16*Parámetros!E8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>Casual</t>
+        </is>
+      </c>
+      <c r="B22" s="7">
+        <f>Calculadora!B27</f>
+        <v/>
+      </c>
+      <c r="C22" s="8">
+        <f>D13*Parámetros!B9+D14*Parámetros!C9+D15*Parámetros!D9+D16*Parámetros!E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>Global (promedio de los 4 vínculos)</t>
+        </is>
+      </c>
+      <c r="B24" s="7">
+        <f>Calculadora!B29</f>
+        <v/>
+      </c>
+      <c r="C24" s="8">
+        <f>AVERAGE(C19:C22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="J30">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(UPPER(B4),"Á","A"),"É","E"),"Í","I"),"Ó","O"),"Ú","U"),"Ü","U"),"Ñ","N")</f>
+        <v/>
+      </c>
+      <c r="P30">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(UPPER(C4),"Á","A"),"É","E"),"Í","I"),"Ó","O"),"Ú","U"),"Ü","U"),"Ñ","N")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="J31">
+        <f>IF(LEN(J30)=0,0,SUMPRODUCT((CODE(MID(J30,ROW(INDIRECT("1:"&amp;LEN(J30))),1))&gt;=65)*(CODE(MID(J30,ROW(INDIRECT("1:"&amp;LEN(J30))),1))&lt;=90)*(MOD(CODE(MID(J30,ROW(INDIRECT("1:"&amp;LEN(J30))),1))-65,9)+1)))</f>
+        <v/>
+      </c>
+      <c r="P31">
+        <f>IF(LEN(P30)=0,0,SUMPRODUCT((CODE(MID(P30,ROW(INDIRECT("1:"&amp;LEN(P30))),1))&gt;=65)*(CODE(MID(P30,ROW(INDIRECT("1:"&amp;LEN(P30))),1))&lt;=90)*(MOD(CODE(MID(P30,ROW(INDIRECT("1:"&amp;LEN(P30))),1))-65,9)+1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="J32">
+        <f>IF(LEN(J30)=0,0,SUMPRODUCT((CODE(MID(J30,ROW(INDIRECT("1:"&amp;LEN(J30))),1))&gt;=65)*(CODE(MID(J30,ROW(INDIRECT("1:"&amp;LEN(J30))),1))&lt;=90)*(MOD(CODE(MID(J30,ROW(INDIRECT("1:"&amp;LEN(J30))),1))-65,9)+1)*ISNUMBER(SEARCH(MID(J30,ROW(INDIRECT("1:"&amp;LEN(J30))),1),"AEIOU"))))</f>
+        <v/>
+      </c>
+      <c r="P32">
+        <f>IF(LEN(P30)=0,0,SUMPRODUCT((CODE(MID(P30,ROW(INDIRECT("1:"&amp;LEN(P30))),1))&gt;=65)*(CODE(MID(P30,ROW(INDIRECT("1:"&amp;LEN(P30))),1))&lt;=90)*(MOD(CODE(MID(P30,ROW(INDIRECT("1:"&amp;LEN(P30))),1))-65,9)+1)*ISNUMBER(SEARCH(MID(P30,ROW(INDIRECT("1:"&amp;LEN(P30))),1),"AEIOU"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="J33">
+        <f>J31-J32</f>
+        <v/>
+      </c>
+      <c r="P33">
+        <f>P31-P32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="J35">
+        <f>(INT(J31/1000)+MOD(INT(J31/100),10)+MOD(INT(J31/10),10)+MOD(J31,10))</f>
+        <v/>
+      </c>
+      <c r="K35">
+        <f>(INT(J35/1000)+MOD(INT(J35/100),10)+MOD(INT(J35/10),10)+MOD(J35,10))</f>
+        <v/>
+      </c>
+      <c r="L35">
+        <f>IF(J31&lt;10,J31,IF(OR(J31=11,J31=22,J31=33),J31,IF(J35&lt;10,J35,IF(OR(J35=11,J35=22,J35=33),J35,IF(K35&lt;10,K35,IF(OR(K35=11,K35=22,K35=33),K35,(INT(K35/1000)+MOD(INT(K35/100),10)+MOD(INT(K35/10),10)+MOD(K35,10))))))))</f>
+        <v/>
+      </c>
+      <c r="P35">
+        <f>(INT(P31/1000)+MOD(INT(P31/100),10)+MOD(INT(P31/10),10)+MOD(P31,10))</f>
+        <v/>
+      </c>
+      <c r="Q35">
+        <f>(INT(P35/1000)+MOD(INT(P35/100),10)+MOD(INT(P35/10),10)+MOD(P35,10))</f>
+        <v/>
+      </c>
+      <c r="R35">
+        <f>IF(P31&lt;10,P31,IF(OR(P31=11,P31=22,P31=33),P31,IF(P35&lt;10,P35,IF(OR(P35=11,P35=22,P35=33),P35,IF(Q35&lt;10,Q35,IF(OR(Q35=11,Q35=22,Q35=33),Q35,(INT(Q35/1000)+MOD(INT(Q35/100),10)+MOD(INT(Q35/10),10)+MOD(Q35,10))))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="J36">
+        <f>(INT(J32/1000)+MOD(INT(J32/100),10)+MOD(INT(J32/10),10)+MOD(J32,10))</f>
+        <v/>
+      </c>
+      <c r="K36">
+        <f>(INT(J36/1000)+MOD(INT(J36/100),10)+MOD(INT(J36/10),10)+MOD(J36,10))</f>
+        <v/>
+      </c>
+      <c r="L36">
+        <f>IF(J32&lt;10,J32,IF(OR(J32=11,J32=22,J32=33),J32,IF(J36&lt;10,J36,IF(OR(J36=11,J36=22,J36=33),J36,IF(K36&lt;10,K36,IF(OR(K36=11,K36=22,K36=33),K36,(INT(K36/1000)+MOD(INT(K36/100),10)+MOD(INT(K36/10),10)+MOD(K36,10))))))))</f>
+        <v/>
+      </c>
+      <c r="P36">
+        <f>(INT(P32/1000)+MOD(INT(P32/100),10)+MOD(INT(P32/10),10)+MOD(P32,10))</f>
+        <v/>
+      </c>
+      <c r="Q36">
+        <f>(INT(P36/1000)+MOD(INT(P36/100),10)+MOD(INT(P36/10),10)+MOD(P36,10))</f>
+        <v/>
+      </c>
+      <c r="R36">
+        <f>IF(P32&lt;10,P32,IF(OR(P32=11,P32=22,P32=33),P32,IF(P36&lt;10,P36,IF(OR(P36=11,P36=22,P36=33),P36,IF(Q36&lt;10,Q36,IF(OR(Q36=11,Q36=22,Q36=33),Q36,(INT(Q36/1000)+MOD(INT(Q36/100),10)+MOD(INT(Q36/10),10)+MOD(Q36,10))))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="J37">
+        <f>(INT(J33/1000)+MOD(INT(J33/100),10)+MOD(INT(J33/10),10)+MOD(J33,10))</f>
+        <v/>
+      </c>
+      <c r="K37">
+        <f>(INT(J37/1000)+MOD(INT(J37/100),10)+MOD(INT(J37/10),10)+MOD(J37,10))</f>
+        <v/>
+      </c>
+      <c r="L37">
+        <f>IF(J33&lt;10,J33,IF(OR(J33=11,J33=22,J33=33),J33,IF(J37&lt;10,J37,IF(OR(J37=11,J37=22,J37=33),J37,IF(K37&lt;10,K37,IF(OR(K37=11,K37=22,K37=33),K37,(INT(K37/1000)+MOD(INT(K37/100),10)+MOD(INT(K37/10),10)+MOD(K37,10))))))))</f>
+        <v/>
+      </c>
+      <c r="P37">
+        <f>(INT(P33/1000)+MOD(INT(P33/100),10)+MOD(INT(P33/10),10)+MOD(P33,10))</f>
+        <v/>
+      </c>
+      <c r="Q37">
+        <f>(INT(P37/1000)+MOD(INT(P37/100),10)+MOD(INT(P37/10),10)+MOD(P37,10))</f>
+        <v/>
+      </c>
+      <c r="R37">
+        <f>IF(P33&lt;10,P33,IF(OR(P33=11,P33=22,P33=33),P33,IF(P37&lt;10,P37,IF(OR(P37=11,P37=22,P37=33),P37,IF(Q37&lt;10,Q37,IF(OR(Q37=11,Q37=22,Q37=33),Q37,(INT(Q37/1000)+MOD(INT(Q37/100),10)+MOD(INT(Q37/10),10)+MOD(Q37,10))))))))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>